<commit_message>
Update GBC 연구논문 DB
</commit_message>
<xml_diff>
--- a/database/GBC_연구논문_DB.xlsx
+++ b/database/GBC_연구논문_DB.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O679"/>
+  <dimension ref="A1:O680"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -51681,6 +51681,88 @@
         </is>
       </c>
     </row>
+    <row r="680">
+      <c r="A680" t="n">
+        <v>679</v>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>Alexander Chernev</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>2003</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>When More Is Less and Less Is More: The Role of Ideal Point Availability and Assortment in Consumer Choice</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>Journal of Consumer Research</t>
+        </is>
+      </c>
+      <c r="F680" t="inlineStr">
+        <is>
+          <t>구성적 선호 관점 (Constructive View of Preferences), 정보 과부하 이론 (Cognitive Overload Theory), 인지부조화 이론 (Cognitive Dissonance Theory)</t>
+        </is>
+      </c>
+      <c r="G680" t="inlineStr">
+        <is>
+          <t>[Product Assortment Size] x [Ideal Point Availability] -&gt; [Preference Strength / Choice Confidence / Switching Propensity / Decision Difficulty]</t>
+        </is>
+      </c>
+      <c r="H680" t="inlineStr">
+        <is>
+          <t>H1: The availability of an articulated ideal point moderates the impact of assortment on consumer preferences. (명확히 표현된 이상점의 이용가능성은 제품 구색이 소비자 선호에 미치는 영향을 조절할 것이다.)
+H2: When choosing from a larger assortment, consumers with an available ideal point are likely to have stronger preferences for the chosen option than consumers without an available ideal attribute combination. (대형 구색에서 선택할 때, 이상점을 이용할 수 있는 소비자는 이상적 속성 조합을 이용할 수 없는 소비자보다 선택한 대안에 대해 더 강한 선호를 가질 것이다.)
+H3: When choosing from a smaller assortment, consumers with an available ideal point are likely to have weaker preferences for the chosen option than consumers without an available ideal attribute combination. (소형 구색에서 선택할 때, 이상점을 이용할 수 있는 소비자는 이상적 속성 조합을 이용할 수 없는 소비자보다 선택한 대안에 대해 더 약한 선호를 가질 것이다.)</t>
+        </is>
+      </c>
+      <c r="I680" t="inlineStr">
+        <is>
+          <t>제품 구색 크기 (Product Assortment Size: Small vs. Large)</t>
+        </is>
+      </c>
+      <c r="J680" t="inlineStr">
+        <is>
+          <t>선호의 강도 (Preference Strength: 전환 행동/의도 Switching Propensity, 결정 확신도 Decision Confidence, 결정 난이도 Decision Difficulty)</t>
+        </is>
+      </c>
+      <c r="K680" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L680" t="inlineStr">
+        <is>
+          <t>이상점 이용가능성 (Ideal Point Availability)</t>
+        </is>
+      </c>
+      <c r="M680" t="inlineStr">
+        <is>
+          <t>제품 구색의 크기가 소비자의 선택 선호 강도에 미치는 영향은 이상점(Ideal Point)의 이용가능성에 의해 조절된다. 대형 구색에서 선택할 때 이상점이 명확히 형성된 소비자는 선택에 대한 확신이 높고 다른 대안으로 전환할 가능성이 낮아 선호 강도가 강화되었으나, 소형 구색에서는 이상점이 형성된 소비자가 구색 내에서 완전한 일치 대안을 찾지 못해 선호 강도가 오히려 약화되는 경향을 보였다.</t>
+        </is>
+      </c>
+      <c r="N680" t="inlineStr">
+        <is>
+          <t>Think about your ideal chocolate. Indicate the most attractive level of each of the attributes describing the choice alternatives and rank order these attributes. / 당신의 이상적인 초콜릿에 대해 생각해보십시오. 선택 대안들을 설명하는 각 속성의 가장 매력적인 수준을 표시하고 이 속성들의 순위를 매기십시오.
+Imagine that you are buying a sofa. Think about what your ideal sofa looks like (e.g., in terms of color, upholstery, back height, cushion softness). Please, describe your ideal sofa in the space below. / 소파를 구매한다고 가정해 보십시오. 당신의 이상적인 소파가 어떤 모습일지 생각해 보십시오(예: 색상, 천/가죽 재질, 등받이 높이, 쿠션의 폭신함 측면에서). 아래 공간에 당신의 이상적인 소파를 기술해 주십시오.
+Choose between a small box containing two chocolates of the exact same kind that you selected in the preceding choice task and a small box containing two of the most popular chocolates from the entire Godiva collection. / 이전 선택 과제에서 선택한 것과 정확히 동일한 종류의 초콜릿 2개가 들어있는 작은 상자와 전체 고디바 컬렉션 중 가장 인기 있는 초콜릿 2개가 들어있는 작은 상자 중 하나를 선택하십시오.
+Imagine that you have to choose between the sofa you just selected and a sofa that has been recommended by the sales associate. Which one would you buy? / 방금 선택한 소파와 판매 직원이 추천한 소파 중에서 선택해야 한다고 가정해 보십시오. 당신은 어떤 것을 구매하시겠습니까?
+How would you rate your confidence that you will actually like the sofa [product] you selected? / 당신이 선택한 소파[제품]를 실제로 마음에 들어 할 것이라는 확신을 어떻게 평가하시겠습니까?
+How would you rate the difficulty of this decision for you? / 이 결정이 당신에게 얼마나 어려웠는지 평가해주십시오.</t>
+        </is>
+      </c>
+      <c r="O680" t="inlineStr">
+        <is>
+          <t>10.1086/376808</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>